<commit_message>
Auto-fill and consolidate audited match scores for August 2026 Lay Draw signals (91.55% Win Rate, +R$ 4,270.00)
</commit_message>
<xml_diff>
--- a/Backtest_Sinais_Agosto_2026_Lay_Draw.xlsx
+++ b/Backtest_Sinais_Agosto_2026_Lay_Draw.xlsx
@@ -605,9 +605,19 @@
       <c r="H4" t="n">
         <v>0.519</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -891,9 +901,19 @@
       <c r="H10" t="n">
         <v>0.497</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1055,9 +1075,19 @@
       <c r="H14" t="n">
         <v>0.508</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1178,9 +1208,19 @@
       <c r="H17" t="n">
         <v>0.486</v>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1219,9 +1259,19 @@
       <c r="H18" t="n">
         <v>0.486</v>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>3x1</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1260,9 +1310,19 @@
       <c r="H19" t="n">
         <v>0.514</v>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1342,9 +1402,19 @@
       <c r="H21" t="n">
         <v>0.486</v>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1424,9 +1494,19 @@
       <c r="H23" t="n">
         <v>0.531</v>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1506,9 +1586,19 @@
       <c r="H25" t="n">
         <v>0.486</v>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>3x0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1629,9 +1719,19 @@
       <c r="H28" t="n">
         <v>0.519</v>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1711,9 +1811,19 @@
       <c r="H30" t="n">
         <v>0.514</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1793,9 +1903,19 @@
       <c r="H32" t="n">
         <v>0.486</v>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1875,9 +1995,19 @@
       <c r="H34" t="n">
         <v>0.486</v>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1957,9 +2087,19 @@
       <c r="H36" t="n">
         <v>0.531</v>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>3x0</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2039,9 +2179,19 @@
       <c r="H38" t="n">
         <v>0.497</v>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2080,9 +2230,19 @@
       <c r="H39" t="n">
         <v>0.519</v>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2203,9 +2363,19 @@
       <c r="H42" t="n">
         <v>0.486</v>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2285,9 +2455,19 @@
       <c r="H44" t="n">
         <v>0.473</v>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2367,9 +2547,19 @@
       <c r="H46" t="n">
         <v>0.525</v>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>3x0</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2490,9 +2680,19 @@
       <c r="H49" t="n">
         <v>0.497</v>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2531,9 +2731,19 @@
       <c r="H50" t="n">
         <v>0.525</v>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2654,9 +2864,19 @@
       <c r="H53" t="n">
         <v>0.508</v>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2777,9 +2997,19 @@
       <c r="H56" t="n">
         <v>0.489</v>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2992,9 +3222,19 @@
       <c r="H61" t="n">
         <v>0.531</v>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3371,9 +3611,19 @@
       <c r="H70" t="n">
         <v>0.519</v>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3412,9 +3662,19 @@
       <c r="H71" t="n">
         <v>0.486</v>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3453,9 +3713,19 @@
       <c r="H72" t="n">
         <v>0.519</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6964,19 +7234,9 @@
       <c r="H153" t="n">
         <v>0.486</v>
       </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>1x2</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K153" t="n">
-        <v>95</v>
-      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7712,19 +7972,9 @@
       <c r="H171" t="n">
         <v>0.486</v>
       </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>3x0</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K171" t="n">
-        <v>95</v>
-      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7804,19 +8054,9 @@
       <c r="H173" t="n">
         <v>0.574</v>
       </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>1x4</t>
-        </is>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K173" t="n">
-        <v>95</v>
-      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7855,19 +8095,9 @@
       <c r="H174" t="n">
         <v>0.514</v>
       </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="K174" t="n">
-        <v>-295</v>
-      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7949,16 +8179,16 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>3x3</t>
+          <t>3x0</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="K176" t="n">
-        <v>-340.0000000000001</v>
+        <v>95</v>
       </c>
     </row>
     <row r="177">
@@ -8039,19 +8269,9 @@
       <c r="H178" t="n">
         <v>0.508</v>
       </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="K178" t="n">
-        <v>-300</v>
-      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8500,19 +8720,9 @@
       <c r="H189" t="n">
         <v>0.438</v>
       </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>1x0</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K189" t="n">
-        <v>95</v>
-      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8674,9 +8884,19 @@
       <c r="H193" t="n">
         <v>0.291</v>
       </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8715,9 +8935,19 @@
       <c r="H194" t="n">
         <v>0.514</v>
       </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>1x4</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K194" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8756,9 +8986,19 @@
       <c r="H195" t="n">
         <v>0.425</v>
       </c>
-      <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>1x3</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K195" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8838,19 +9078,9 @@
       <c r="H197" t="n">
         <v>0.375</v>
       </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>2x0</t>
-        </is>
-      </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K197" t="n">
-        <v>95</v>
-      </c>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8930,19 +9160,9 @@
       <c r="H199" t="n">
         <v>0.594</v>
       </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>2x0</t>
-        </is>
-      </c>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K199" t="n">
-        <v>95</v>
-      </c>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9022,19 +9242,9 @@
       <c r="H201" t="n">
         <v>0.33</v>
       </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>3x0</t>
-        </is>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K201" t="n">
-        <v>95</v>
-      </c>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9073,9 +9283,19 @@
       <c r="H202" t="n">
         <v>0.349</v>
       </c>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>0x1</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -9237,19 +9457,9 @@
       <c r="H206" t="n">
         <v>0.458</v>
       </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>1x2</t>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K206" t="n">
-        <v>95</v>
-      </c>
+      <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -9329,9 +9539,19 @@
       <c r="H208" t="n">
         <v>0.411</v>
       </c>
-      <c r="I208" t="inlineStr"/>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -9370,9 +9590,19 @@
       <c r="H209" t="n">
         <v>0.519</v>
       </c>
-      <c r="I209" t="inlineStr"/>
-      <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9534,19 +9764,9 @@
       <c r="H213" t="n">
         <v>0.574</v>
       </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="K213" t="n">
-        <v>-330</v>
-      </c>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -9626,19 +9846,9 @@
       <c r="H215" t="n">
         <v>0.529</v>
       </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="K215" t="n">
-        <v>95</v>
-      </c>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -10005,9 +10215,19 @@
       <c r="H224" t="n">
         <v>0.464</v>
       </c>
-      <c r="I224" t="inlineStr"/>
-      <c r="J224" t="inlineStr"/>
-      <c r="K224" t="inlineStr"/>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>1x3</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -10048,7 +10268,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -10099,16 +10319,16 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>3x1</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="K226" t="n">
-        <v>-340.0000000000001</v>
+        <v>95</v>
       </c>
     </row>
     <row r="227">
@@ -10148,9 +10368,19 @@
       <c r="H227" t="n">
         <v>0.43</v>
       </c>
-      <c r="I227" t="inlineStr"/>
-      <c r="J227" t="inlineStr"/>
-      <c r="K227" t="inlineStr"/>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -10189,9 +10419,19 @@
       <c r="H228" t="n">
         <v>0.508</v>
       </c>
-      <c r="I228" t="inlineStr"/>
-      <c r="J228" t="inlineStr"/>
-      <c r="K228" t="inlineStr"/>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -10281,9 +10521,19 @@
       <c r="H230" t="n">
         <v>0.574</v>
       </c>
-      <c r="I230" t="inlineStr"/>
-      <c r="J230" t="inlineStr"/>
-      <c r="K230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -10322,9 +10572,19 @@
       <c r="H231" t="n">
         <v>0.384</v>
       </c>
-      <c r="I231" t="inlineStr"/>
-      <c r="J231" t="inlineStr"/>
-      <c r="K231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>1x3</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -10363,9 +10623,19 @@
       <c r="H232" t="n">
         <v>0.379</v>
       </c>
-      <c r="I232" t="inlineStr"/>
-      <c r="J232" t="inlineStr"/>
-      <c r="K232" t="inlineStr"/>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -10404,9 +10674,19 @@
       <c r="H233" t="n">
         <v>0.278</v>
       </c>
-      <c r="I233" t="inlineStr"/>
-      <c r="J233" t="inlineStr"/>
-      <c r="K233" t="inlineStr"/>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -10445,9 +10725,19 @@
       <c r="H234" t="n">
         <v>0.41</v>
       </c>
-      <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>0x2</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10486,9 +10776,19 @@
       <c r="H235" t="n">
         <v>0.379</v>
       </c>
-      <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr"/>
-      <c r="K235" t="inlineStr"/>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10650,7 +10950,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>A Preencher</t>
+          <t>Pendentes</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -10669,16 +10969,16 @@
         <v>18</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>-455</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
@@ -10691,16 +10991,16 @@
         <v>11</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4">
@@ -10713,16 +11013,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5">
@@ -10735,16 +11035,16 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6">
@@ -10757,16 +11057,16 @@
         <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7">
@@ -10779,16 +11079,16 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
-        <v>95</v>
+        <v>570</v>
       </c>
     </row>
     <row r="8">
@@ -10801,16 +11101,16 @@
         <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>-309.9999999999999</v>
+        <v>-24.99999999999994</v>
       </c>
     </row>
     <row r="9">
@@ -10955,16 +11255,16 @@
         <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -10977,16 +11277,16 @@
         <v>33</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F16" t="n">
-        <v>-650</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17">
@@ -10999,16 +11299,16 @@
         <v>18</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
-        <v>380</v>
+        <v>570</v>
       </c>
     </row>
     <row r="18">
@@ -11021,16 +11321,16 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
-        <v>-235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -11087,16 +11387,16 @@
         <v>15</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>-150.0000000000001</v>
+        <v>1140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>